<commit_message>
Plotting a "max capacity utill target is reached" strategy against the optimal
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/annual analysis/results_summary.xlsx
+++ b/tutorials/flex_ro/annual analysis/results_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\annual analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A942D8E-0C0F-4115-9E5C-464FB2E56ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A14CBA-416A-4676-A28D-DE4166F7A32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,11 +35,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}</author>
+  </authors>
+  <commentList>
+    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This does include the one month of shutdown at the end of the year</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
-  <si>
-    <t>Scenario</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="16">
   <si>
     <t>Dry</t>
   </si>
@@ -74,29 +89,38 @@
     <t>Normalized Cost ($/AF)</t>
   </si>
   <si>
-    <t>Sum</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Running Total</t>
-  </si>
-  <si>
-    <t>Count</t>
+    <t>Rain Year Type</t>
+  </si>
+  <si>
+    <t>Production Strat</t>
+  </si>
+  <si>
+    <t>Flex</t>
+  </si>
+  <si>
+    <t>Max Out</t>
+  </si>
+  <si>
+    <t>NR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -143,16 +167,23 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Churchill, Jake" id="{FB552105-D09F-4C39-A3B7-87EBDEB6DC39}" userId="S::rchurchi@nrel.gov::24b6a320-1211-4379-9513-990e66715a0d" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}" name="Table1" displayName="Table1" ref="A1:H10" totalsRowShown="0">
-  <autoFilter ref="A1:H10" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1CF06523-CCC8-4FEF-A4D1-4CF85579D0DE}" name="Scenario"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}" name="Table1" displayName="Table1" ref="A1:I12" totalsRowShown="0">
+  <autoFilter ref="A1:I12" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{1CF06523-CCC8-4FEF-A4D1-4CF85579D0DE}" name="Rain Year Type"/>
+    <tableColumn id="9" xr3:uid="{4ADE17F0-D4B7-4A06-B940-2A90184BA957}" name="Production Strat"/>
     <tableColumn id="2" xr3:uid="{8D74FC59-D61B-41FE-B59B-DFCECF68DE49}" name="Target AF"/>
     <tableColumn id="3" xr3:uid="{3764D810-7709-4D52-B48F-CCD0EE55641B}" name="Total AF"/>
     <tableColumn id="4" xr3:uid="{A02BCB72-5C8F-4D42-8DE8-C41F1EE5D781}" name="Total Op Cost"/>
     <tableColumn id="5" xr3:uid="{B4E06B85-A541-4975-95A8-E875BF60AE6E}" name="Normalized Cost ($/AF)" dataDxfId="0">
-      <calculatedColumnFormula>D2/C2</calculatedColumnFormula>
+      <calculatedColumnFormula>E2/D2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{CB888B5D-70EC-4307-AAAA-04DB24B04060}" name="Q1 Water"/>
     <tableColumn id="7" xr3:uid="{3CF28664-7840-45C8-AB81-50412EE444EE}" name="Q2 Water"/>
@@ -423,267 +454,390 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A4" dT="2026-09-30T22:23:34.00" personId="{FB552105-D09F-4C39-A3B7-87EBDEB6DC39}" id="{0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}">
+    <text>This does include the one month of shutdown at the end of the year</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.15234375" customWidth="1"/>
-    <col min="2" max="2" width="13.921875" customWidth="1"/>
-    <col min="4" max="4" width="12.53515625" customWidth="1"/>
-    <col min="5" max="5" width="21.3046875" customWidth="1"/>
-    <col min="6" max="8" width="9.53515625" customWidth="1"/>
+    <col min="1" max="2" width="22.26953125" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" customWidth="1"/>
+    <col min="5" max="5" width="12.54296875" customWidth="1"/>
+    <col min="6" max="6" width="21.26953125" customWidth="1"/>
+    <col min="7" max="9" width="9.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
+        <v>10000</v>
+      </c>
+      <c r="D2">
+        <v>10000</v>
+      </c>
+      <c r="E2">
+        <v>5085642</v>
+      </c>
+      <c r="F2" s="1">
+        <f>E2/D2</f>
+        <v>508.56420000000003</v>
+      </c>
+      <c r="G2">
+        <v>2510</v>
+      </c>
+      <c r="H2">
+        <v>5075</v>
+      </c>
+      <c r="I2">
+        <v>7709</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>10000</v>
-      </c>
-      <c r="C2">
-        <v>10000</v>
-      </c>
-      <c r="D2">
-        <v>5085642</v>
-      </c>
-      <c r="E2" s="1">
-        <f>D2/C2</f>
-        <v>508.56420000000003</v>
-      </c>
-      <c r="F2">
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>10000</v>
+      </c>
+      <c r="D3">
+        <v>10000</v>
+      </c>
+      <c r="E3">
+        <v>5155722</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F9" si="0">E3/D3</f>
+        <v>515.57219999999995</v>
+      </c>
+      <c r="G3">
         <v>2510</v>
       </c>
-      <c r="G2">
-        <v>5075</v>
-      </c>
-      <c r="H2">
-        <v>7709</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="H3">
+        <v>4262</v>
+      </c>
+      <c r="I3">
+        <v>7122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>10000</v>
-      </c>
-      <c r="C3">
-        <v>10000</v>
-      </c>
-      <c r="D3">
-        <v>5155722</v>
-      </c>
-      <c r="E3" s="1">
-        <f t="shared" ref="E3:E10" si="0">D3/C3</f>
-        <v>515.57219999999995</v>
-      </c>
-      <c r="F3">
-        <v>2510</v>
-      </c>
-      <c r="G3">
-        <v>4262</v>
-      </c>
-      <c r="H3">
-        <v>7122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>10000</v>
+      <c r="B4" t="s">
+        <v>13</v>
       </c>
       <c r="C4">
         <v>10000</v>
       </c>
       <c r="D4">
+        <v>10000</v>
+      </c>
+      <c r="E4">
         <v>5297867</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <f t="shared" si="0"/>
         <v>529.7867</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>3062</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>4342</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>5942</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>10000</v>
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
       </c>
       <c r="C5">
+        <v>10000</v>
+      </c>
+      <c r="D5">
         <v>9600</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>5136438</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <f t="shared" si="0"/>
         <v>535.04562499999997</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>4160</v>
-      </c>
-      <c r="G5">
-        <v>5440</v>
       </c>
       <c r="H5">
         <v>5440</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="I5">
+        <v>5440</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <v>8000</v>
+      </c>
+      <c r="D6">
+        <v>8000</v>
+      </c>
+      <c r="E6">
+        <v>4120082</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+        <v>515.01025000000004</v>
+      </c>
+      <c r="G6">
+        <v>1196</v>
+      </c>
+      <c r="H6">
+        <v>3723</v>
+      </c>
+      <c r="I6">
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7">
-        <v>8000</v>
+      <c r="B7" t="s">
+        <v>13</v>
       </c>
       <c r="C7">
         <v>8000</v>
       </c>
       <c r="D7">
-        <v>4120082</v>
-      </c>
-      <c r="E7" s="1">
+        <v>8000</v>
+      </c>
+      <c r="E7">
+        <v>4142428</v>
+      </c>
+      <c r="F7" s="1">
         <f t="shared" si="0"/>
-        <v>515.01025000000004</v>
-      </c>
-      <c r="F7">
-        <v>1196</v>
+        <v>517.80349999999999</v>
       </c>
       <c r="G7">
-        <v>3723</v>
+        <v>2510</v>
       </c>
       <c r="H7">
-        <v>6250</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+        <v>4269</v>
+      </c>
+      <c r="I7">
+        <v>6037</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
-      <c r="B8">
-        <v>8000</v>
+      <c r="B8" t="s">
+        <v>13</v>
       </c>
       <c r="C8">
         <v>8000</v>
       </c>
       <c r="D8">
-        <v>4142428</v>
-      </c>
-      <c r="E8" s="1">
+        <v>8000</v>
+      </c>
+      <c r="E8">
+        <v>4222268</v>
+      </c>
+      <c r="F8" s="1">
         <f t="shared" si="0"/>
-        <v>517.80349999999999</v>
-      </c>
-      <c r="F8">
+        <v>527.7835</v>
+      </c>
+      <c r="G8">
         <v>2510</v>
       </c>
-      <c r="G8">
-        <v>4269</v>
-      </c>
       <c r="H8">
-        <v>6037</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+        <v>3554</v>
+      </c>
+      <c r="I8">
+        <v>5139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9">
-        <v>8000</v>
+      <c r="B9" t="s">
+        <v>13</v>
       </c>
       <c r="C9">
         <v>8000</v>
       </c>
       <c r="D9">
-        <v>4222268</v>
-      </c>
-      <c r="E9" s="1">
-        <f t="shared" si="0"/>
-        <v>527.7835</v>
-      </c>
-      <c r="F9">
-        <v>2510</v>
-      </c>
-      <c r="G9">
-        <v>3554</v>
-      </c>
-      <c r="H9">
-        <v>5139</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10">
         <v>8000</v>
       </c>
-      <c r="C10">
-        <v>8000</v>
-      </c>
-      <c r="D10">
+      <c r="E9">
         <v>4271851</v>
       </c>
-      <c r="E10" s="1">
+      <c r="F9" s="1">
         <f t="shared" si="0"/>
         <v>533.98137499999996</v>
       </c>
-      <c r="F10">
+      <c r="G9">
         <v>3840</v>
       </c>
-      <c r="G10">
+      <c r="H9">
         <v>5120</v>
       </c>
+      <c r="I9">
+        <v>5120</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10">
+        <v>10000</v>
+      </c>
+      <c r="D10">
+        <v>10000</v>
+      </c>
+      <c r="E10">
+        <v>5291617</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" ref="F10:F12" si="1">E10/D10</f>
+        <v>529.1617</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
       <c r="H10">
-        <v>5120</v>
+        <v>8319</v>
+      </c>
+      <c r="I10">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11">
+        <v>10000</v>
+      </c>
+      <c r="D11">
+        <v>10000</v>
+      </c>
+      <c r="E11">
+        <v>5297275</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="1"/>
+        <v>529.72749999999996</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11">
+        <v>7039</v>
+      </c>
+      <c r="I11">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12">
+        <v>10000</v>
+      </c>
+      <c r="D12">
+        <v>10000</v>
+      </c>
+      <c r="E12">
+        <v>5297552</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="1"/>
+        <v>529.75519999999995</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12">
+        <v>5439</v>
+      </c>
+      <c r="I12" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Updating annual analysis script and plots
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/annual analysis/results_summary.xlsx
+++ b/tutorials/flex_ro/annual analysis/results_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\annual analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A14CBA-416A-4676-A28D-DE4166F7A32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89008BC4-CE7F-4484-914F-422562B2C3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
     <author>tc={0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}</author>
   </authors>
   <commentList>
-    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="17">
   <si>
     <t>Dry</t>
   </si>
@@ -102,12 +102,18 @@
   </si>
   <si>
     <t>NR</t>
+  </si>
+  <si>
+    <t>Op Cost (M$)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -117,10 +123,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -143,14 +150,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -174,15 +186,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}" name="Table1" displayName="Table1" ref="A1:I12" totalsRowShown="0">
-  <autoFilter ref="A1:I12" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}" name="Table1" displayName="Table1" ref="A1:J12" totalsRowShown="0">
+  <autoFilter ref="A1:J12" xr:uid="{3014DECB-E5FE-4EE4-BF8D-FF4A37CA9401}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Dry"/>
+        <filter val="Normal"/>
+        <filter val="Wet"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="10000"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J12">
+    <sortCondition ref="A1:A12"/>
+  </sortState>
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1CF06523-CCC8-4FEF-A4D1-4CF85579D0DE}" name="Rain Year Type"/>
     <tableColumn id="9" xr3:uid="{4ADE17F0-D4B7-4A06-B940-2A90184BA957}" name="Production Strat"/>
     <tableColumn id="2" xr3:uid="{8D74FC59-D61B-41FE-B59B-DFCECF68DE49}" name="Target AF"/>
     <tableColumn id="3" xr3:uid="{3764D810-7709-4D52-B48F-CCD0EE55641B}" name="Total AF"/>
     <tableColumn id="4" xr3:uid="{A02BCB72-5C8F-4D42-8DE8-C41F1EE5D781}" name="Total Op Cost"/>
-    <tableColumn id="5" xr3:uid="{B4E06B85-A541-4975-95A8-E875BF60AE6E}" name="Normalized Cost ($/AF)" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{4EFEBA91-72E5-4FBE-9F3D-E5DFA5C158E5}" name="Op Cost (M$)" dataDxfId="0">
+      <calculatedColumnFormula>Table1[[#This Row],[Total Op Cost]]/10^6</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{B4E06B85-A541-4975-95A8-E875BF60AE6E}" name="Normalized Cost ($/AF)" dataDxfId="1">
       <calculatedColumnFormula>E2/D2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{CB888B5D-70EC-4307-AAAA-04DB24B04060}" name="Q1 Water"/>
@@ -456,7 +487,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A4" dT="2026-09-30T22:23:34.00" personId="{FB552105-D09F-4C39-A3B7-87EBDEB6DC39}" id="{0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}">
+  <threadedComment ref="A10" dT="2026-09-30T22:23:34.00" personId="{FB552105-D09F-4C39-A3B7-87EBDEB6DC39}" id="{0C0135B7-E1FB-4B9D-A926-3B25F418FE0C}">
     <text>This does include the one month of shutdown at the end of the year</text>
   </threadedComment>
 </ThreadedComments>
@@ -464,17 +495,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="22.26953125" customWidth="1"/>
-    <col min="3" max="3" width="13.90625" customWidth="1"/>
-    <col min="5" max="5" width="12.54296875" customWidth="1"/>
-    <col min="6" max="6" width="21.26953125" customWidth="1"/>
-    <col min="7" max="9" width="9.54296875" customWidth="1"/>
+    <col min="1" max="2" width="22.23046875" customWidth="1"/>
+    <col min="3" max="3" width="13.921875" customWidth="1"/>
+    <col min="5" max="6" width="12.53515625" customWidth="1"/>
+    <col min="7" max="7" width="21.23046875" customWidth="1"/>
+    <col min="8" max="10" width="9.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -491,20 +522,23 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
@@ -519,53 +553,61 @@
       <c r="E2">
         <v>5085642</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.085642</v>
+      </c>
+      <c r="G2" s="1">
         <f>E2/D2</f>
         <v>508.56420000000003</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>2510</v>
       </c>
-      <c r="H2">
-        <v>5075</v>
-      </c>
       <c r="I2">
-        <v>7709</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+        <v>5333</v>
+      </c>
+      <c r="J2">
+        <v>8095</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
+        <v>10000</v>
+      </c>
+      <c r="D3">
+        <v>10000</v>
+      </c>
+      <c r="E3">
+        <v>5291617</v>
+      </c>
+      <c r="F3" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.2916169999999996</v>
+      </c>
+      <c r="G3" s="1">
+        <f>E3/D3</f>
+        <v>529.1617</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3">
+        <v>8319</v>
+      </c>
+      <c r="J3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>10000</v>
-      </c>
-      <c r="D3">
-        <v>10000</v>
-      </c>
-      <c r="E3">
-        <v>5155722</v>
-      </c>
-      <c r="F3" s="1">
-        <f t="shared" ref="F3:F9" si="0">E3/D3</f>
-        <v>515.57219999999995</v>
-      </c>
-      <c r="G3">
-        <v>2510</v>
-      </c>
-      <c r="H3">
-        <v>4262</v>
-      </c>
-      <c r="I3">
-        <v>7122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -577,54 +619,62 @@
         <v>10000</v>
       </c>
       <c r="E4">
-        <v>5297867</v>
-      </c>
-      <c r="F4" s="1">
-        <f t="shared" si="0"/>
-        <v>529.7867</v>
-      </c>
-      <c r="G4">
-        <v>3062</v>
+        <v>5155722</v>
+      </c>
+      <c r="F4" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.1557219999999999</v>
+      </c>
+      <c r="G4" s="1">
+        <f>E4/D4</f>
+        <v>515.57219999999995</v>
       </c>
       <c r="H4">
-        <v>4342</v>
+        <v>2510</v>
       </c>
       <c r="I4">
-        <v>5942</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+        <v>5005</v>
+      </c>
+      <c r="J4">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <v>10000</v>
       </c>
       <c r="D5">
-        <v>9600</v>
+        <v>10000</v>
       </c>
       <c r="E5">
-        <v>5136438</v>
-      </c>
-      <c r="F5" s="1">
-        <f t="shared" si="0"/>
-        <v>535.04562499999997</v>
-      </c>
-      <c r="G5">
-        <v>4160</v>
-      </c>
-      <c r="H5">
-        <v>5440</v>
+        <v>5297275</v>
+      </c>
+      <c r="F5" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.297275</v>
+      </c>
+      <c r="G5" s="1">
+        <f>E5/D5</f>
+        <v>529.72749999999996</v>
+      </c>
+      <c r="H5" t="s">
+        <v>15</v>
       </c>
       <c r="I5">
-        <v>5440</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+        <v>7039</v>
+      </c>
+      <c r="J5">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B6" t="s">
@@ -639,22 +689,26 @@
       <c r="E6">
         <v>4120082</v>
       </c>
-      <c r="F6" s="1">
-        <f t="shared" si="0"/>
+      <c r="F6">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>4.120082</v>
+      </c>
+      <c r="G6" s="1">
+        <f>E6/D6</f>
         <v>515.01025000000004</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>1196</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>3723</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>6250</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B7" t="s">
@@ -667,24 +721,28 @@
         <v>8000</v>
       </c>
       <c r="E7">
-        <v>4142428</v>
-      </c>
-      <c r="F7" s="1">
-        <f t="shared" si="0"/>
-        <v>517.80349999999999</v>
-      </c>
-      <c r="G7">
+        <v>4143428</v>
+      </c>
+      <c r="F7">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>4.1434280000000001</v>
+      </c>
+      <c r="G7" s="1">
+        <f>E7/D7</f>
+        <v>517.92849999999999</v>
+      </c>
+      <c r="H7">
         <v>2510</v>
       </c>
-      <c r="H7">
-        <v>4269</v>
-      </c>
       <c r="I7">
-        <v>6037</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+        <v>4340</v>
+      </c>
+      <c r="J7">
+        <v>6170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B8" t="s">
@@ -699,22 +757,26 @@
       <c r="E8">
         <v>4222268</v>
       </c>
-      <c r="F8" s="1">
-        <f t="shared" si="0"/>
+      <c r="F8">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>4.2222679999999997</v>
+      </c>
+      <c r="G8" s="1">
+        <f>E8/D8</f>
         <v>527.7835</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>2510</v>
       </c>
-      <c r="H8">
-        <v>3554</v>
-      </c>
       <c r="I8">
-        <v>5139</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+        <v>3689</v>
+      </c>
+      <c r="J8">
+        <v>5257</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B9" t="s">
@@ -729,26 +791,30 @@
       <c r="E9">
         <v>4271851</v>
       </c>
-      <c r="F9" s="1">
-        <f t="shared" si="0"/>
+      <c r="F9">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>4.2718509999999998</v>
+      </c>
+      <c r="G9" s="1">
+        <f>E9/D9</f>
         <v>533.98137499999996</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>3840</v>
-      </c>
-      <c r="H9">
-        <v>5120</v>
       </c>
       <c r="I9">
         <v>5120</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>0</v>
+      <c r="J9">
+        <v>5120</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10">
         <v>10000</v>
@@ -757,53 +823,61 @@
         <v>10000</v>
       </c>
       <c r="E10">
-        <v>5291617</v>
-      </c>
-      <c r="F10" s="1">
-        <f t="shared" ref="F10:F12" si="1">E10/D10</f>
-        <v>529.1617</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
+        <v>5210410</v>
+      </c>
+      <c r="F10" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.2104100000000004</v>
+      </c>
+      <c r="G10" s="1">
+        <f>E10/D10</f>
+        <v>521.04100000000005</v>
       </c>
       <c r="H10">
-        <v>8319</v>
+        <v>3062</v>
       </c>
       <c r="I10">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>1</v>
+        <v>4342</v>
+      </c>
+      <c r="J10">
+        <v>5942</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>10000</v>
       </c>
       <c r="D11">
-        <v>10000</v>
+        <v>9600</v>
       </c>
       <c r="E11">
-        <v>5297275</v>
-      </c>
-      <c r="F11" s="1">
-        <f t="shared" si="1"/>
-        <v>529.72749999999996</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
+        <v>5224853</v>
+      </c>
+      <c r="F11" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.2248530000000004</v>
+      </c>
+      <c r="G11" s="1">
+        <f>E11/D11</f>
+        <v>544.25552083333332</v>
       </c>
       <c r="H11">
-        <v>7039</v>
+        <v>4160</v>
       </c>
       <c r="I11">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+        <v>5440</v>
+      </c>
+      <c r="J11">
+        <v>5440</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -819,17 +893,21 @@
       <c r="E12">
         <v>5297552</v>
       </c>
-      <c r="F12" s="1">
-        <f t="shared" si="1"/>
+      <c r="F12" s="3">
+        <f>Table1[[#This Row],[Total Op Cost]]/10^6</f>
+        <v>5.2975519999999996</v>
+      </c>
+      <c r="G12" s="1">
+        <f>E12/D12</f>
         <v>529.75519999999995</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>15</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>5439</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>